<commit_message>
Publish IG v1.0.1 (IG Publisher: 0 errors, 0 broken links)
</commit_message>
<xml_diff>
--- a/CodeSystem-dysphagia-scales-temp.xlsx
+++ b/CodeSystem-dysphagia-scales-temp.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>1.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-28T10:20:05+00:00</t>
+    <t>2026-07-28T10:50:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Publish IG v1.1.0 (IG Publisher: 0 errors, 0 broken links)
</commit_message>
<xml_diff>
--- a/CodeSystem-dysphagia-scales-temp.xlsx
+++ b/CodeSystem-dysphagia-scales-temp.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="54">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.1</t>
+    <t>1.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-28T10:50:36+00:00</t>
+    <t>2026-07-29T08:35:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>Copyright</t>
+  </si>
+  <si>
+    <t>MIT (© 2026 N. Kapan Tunçer and S. Tunçer). These are locally minted placeholder identifiers only. They name validated instruments whose own copyright rests with their developers; no instrument content, scoring rule or item text is reproduced here. The codes are temporary and are expected to be retired once equivalent concepts exist in LOINC or SNOMED CT.</t>
   </si>
   <si>
     <t>Case Sensitive</t>
@@ -410,11 +413,13 @@
       <c r="A13" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="B13" s="2"/>
+      <c r="B13" t="s" s="2">
+        <v>24</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s" s="2">
         <v>13</v>
@@ -422,48 +427,48 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -478,99 +483,99 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D8" s="2"/>
     </row>

</xml_diff>

<commit_message>
Publish IG v1.1.1 (IG Publisher: 0 errors, 0 broken links)
</commit_message>
<xml_diff>
--- a/CodeSystem-dysphagia-scales-temp.xlsx
+++ b/CodeSystem-dysphagia-scales-temp.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.0</t>
+    <t>1.1.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-29T08:35:16+00:00</t>
+    <t>2026-07-29T12:05:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Publish IG v1.2.0 (aspiration-risk flag pattern on CodeableConcept; IG Publisher 0 errors)
</commit_message>
<xml_diff>
--- a/CodeSystem-dysphagia-scales-temp.xlsx
+++ b/CodeSystem-dysphagia-scales-temp.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.1</t>
+    <t>1.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-29T12:05:46+00:00</t>
+    <t>2026-07-31T09:21:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Publish IG v1.2.1 (licence notices on the conformance resources; 0 errors)
</commit_message>
<xml_diff>
--- a/CodeSystem-dysphagia-scales-temp.xlsx
+++ b/CodeSystem-dysphagia-scales-temp.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.0</t>
+    <t>1.2.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-31T09:21:13+00:00</t>
+    <t>2026-08-13T14:00:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>